<commit_message>
Tablas_Stock archivo v2 - May-2026
</commit_message>
<xml_diff>
--- a/Tablas/Tablas_Stock_2026_05.xlsx
+++ b/Tablas/Tablas_Stock_2026_05.xlsx
@@ -1196,17 +1196,17 @@
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>Cierre bajo - Vehículo mal estacionado</t>
+          <t>Cierre bajo - Vehiculo mal estacionado</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr">
         <is>
-          <t>0% (22 casos)</t>
+          <t>22 casos, 0% cierre</t>
         </is>
       </c>
       <c r="F18" s="3" t="inlineStr">
         <is>
-          <t>Tipo 'Vehículo mal estacionado': 22 casos en May-2026 con 0% de cierre (tablero). Cierre muy por debajo del resto del area.</t>
+          <t>Tipo 'Vehiculo mal estacionado': 22 casos en May-2026 que se registran en estado 'Sin asignar' (no se cierran), igual que en abril. Tipo implementado desde marzo 2026. No es demora operativa: revisar con el area si se estan siguiendo los protocolos de implementacion del proceso para tratar este tipo de reclamos.</t>
         </is>
       </c>
     </row>

</xml_diff>